<commit_message>
chore(media): update sample bill payment Excel file
</commit_message>
<xml_diff>
--- a/public/uploads/media/default/sample_bill_payment.xlsx
+++ b/public/uploads/media/default/sample_bill_payment.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moham\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moham\Desktop\Mohamed\Amanah Insurance\ekstrabooks-v2.0\public\uploads\media\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E0E5417-B6E3-49B1-8887-B9DDA1212EE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69CD2C9A-20CB-4F1A-874B-0CB03E789C71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DF11F86E-223F-4DA1-8B0D-8115EA6778EA}"/>
   </bookViews>
@@ -44,9 +44,6 @@
     <t>bill_number</t>
   </si>
   <si>
-    <t>purchase_date</t>
-  </si>
-  <si>
     <t>payment_account</t>
   </si>
   <si>
@@ -57,6 +54,9 @@
   </si>
   <si>
     <t>amount</t>
+  </si>
+  <si>
+    <t>payment_date</t>
   </si>
 </sst>
 </file>
@@ -456,19 +456,19 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(storage): add scoped attachment storage with signed download support
- add `storage_settings` model/migrations and extend attachments with disk, visibility, mime type, and file size fields
- introduce storage services to resolve scope-based settings and store uploads on `public`, `s3`, or `gcs`
- refactor attachment upload handling in billing/invoice/purchase/subcontract/payment flows to use `AttachmentStorageService`
- add signed attachment download route and expose `download_url` for frontend attachment links
- add admin storage settings UI with save/test connection actions and toast notifications
- update filesystem/env config and composer deps for S3/GCS support
- refresh default sample spreadsheet files
</commit_message>
<xml_diff>
--- a/public/uploads/media/default/sample_bill_payment.xlsx
+++ b/public/uploads/media/default/sample_bill_payment.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moham\Desktop\Mohamed\Amanah Insurance\ekstrabooks-v2.0\public\uploads\media\default\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moham\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69CD2C9A-20CB-4F1A-874B-0CB03E789C71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03407B27-B085-49D4-91CD-AF805803935D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DF11F86E-223F-4DA1-8B0D-8115EA6778EA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>supplier_name</t>
   </si>
@@ -56,7 +56,22 @@
     <t>amount</t>
   </si>
   <si>
+    <t>CTT TRAVEL AGENCY</t>
+  </si>
+  <si>
     <t>payment_date</t>
+  </si>
+  <si>
+    <t>Cash Account</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>Bank</t>
+  </si>
+  <si>
+    <t>Equity Bank Account USD</t>
   </si>
 </sst>
 </file>
@@ -98,9 +113,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -435,16 +451,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E16A8DBB-17B5-4635-89F7-2C1D6A512F41}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.85546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="14.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
@@ -459,7 +475,7 @@
         <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
@@ -469,6 +485,52 @@
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1725</v>
+      </c>
+      <c r="C2" s="1">
+        <v>291</v>
+      </c>
+      <c r="D2" s="2">
+        <v>46090</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="1">
+        <v>567577866</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1725</v>
+      </c>
+      <c r="C3" s="1">
+        <v>515.54999999999995</v>
+      </c>
+      <c r="D3" s="2">
+        <v>46091</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="1">
+        <v>567567567</v>
       </c>
     </row>
   </sheetData>

</xml_diff>